<commit_message>
Excel: sayfa adını düzelt, fatura tarihlerini tarih biçimine çevir
- "Fatura_Takip_Dashboard.xlsx" sayfasının adı "Dashboard" yapıldı
- Fatura_Tarihi sütunu metinden tarih biçimine çevrildi
- Fatura_Takip sayfasındaki tekrar eden KPI hesapları kaldırıldı (Dashboard sayfası aynı değerleri hesaplıyor)
</commit_message>
<xml_diff>
--- a/03-Excel-Invoice-Tracking-Dashboard/Invoice_Tracking_Dashboard.xlsx
+++ b/03-Excel-Invoice-Tracking-Dashboard/Invoice_Tracking_Dashboard.xlsx
@@ -15,7 +15,7 @@
   <sheets>
     <sheet name="Pivot_Musteri" sheetId="3" r:id="rId1"/>
     <sheet name="Pivot_Kategori" sheetId="4" r:id="rId2"/>
-    <sheet name="Fatura_Takip_Dashboard.xlsx" sheetId="5" r:id="rId3"/>
+    <sheet name="Dashboard" sheetId="5" r:id="rId3"/>
     <sheet name="Fatura_Takip" sheetId="1" r:id="rId4"/>
     <sheet name="Müşteri_Bilgileri" sheetId="2" r:id="rId5"/>
   </sheets>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="52">
   <si>
     <t>Fatura_ID</t>
   </si>
@@ -6670,7 +6670,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56EAC575-E7A5-48DB-A715-82261278439D}">
-  <dimension ref="A1:P7"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
@@ -6682,13 +6682,9 @@
     <col min="7" max="7" width="15.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="20.28515625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="21.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -6722,22 +6718,13 @@
       <c r="K1" t="s">
         <v>46</v>
       </c>
-      <c r="L1" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="N1" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="P1" s="5" t="s">
-        <v>38</v>
-      </c>
     </row>
-    <row r="2" spans="1:16" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>26</v>
       </c>
-      <c r="B2" t="s">
-        <v>27</v>
+      <c r="B2" s="2">
+        <v>46254</v>
       </c>
       <c r="C2" t="s">
         <v>9</v>
@@ -6769,25 +6756,13 @@
         <f t="shared" ref="K2:K7" ca="1" si="1">IF(I2="Ödendi","Kapandı",IF(H2&lt;TODAY(),"Gecikmiş","Bekliyor"))</f>
         <v>Kapandı</v>
       </c>
-      <c r="L2" s="6">
-        <f>SUM(Table1[Toplam_Tutar])</f>
-        <v>32500</v>
-      </c>
-      <c r="N2" s="7">
-        <f ca="1">SUMIFS(G2:G7,H2:H7,"&lt;"&amp;TODAY(),I2:I7,"Bekliyor")</f>
-        <v>23000</v>
-      </c>
-      <c r="P2" s="7">
-        <f>AVERAGE(Table1[Toplam_Tutar])</f>
-        <v>5416.666666666667</v>
-      </c>
     </row>
-    <row r="3" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>12</v>
       </c>
-      <c r="B3" t="s">
-        <v>28</v>
+      <c r="B3" s="2">
+        <v>46256</v>
       </c>
       <c r="C3" t="s">
         <v>13</v>
@@ -6820,12 +6795,12 @@
         <v>Gecikmiş</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>16</v>
       </c>
-      <c r="B4" t="s">
-        <v>29</v>
+      <c r="B4" s="2">
+        <v>46258</v>
       </c>
       <c r="C4" t="s">
         <v>17</v>
@@ -6857,25 +6832,13 @@
         <f t="shared" ca="1" si="1"/>
         <v>Bekliyor</v>
       </c>
-      <c r="L4" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="M4" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="N4" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="P4" s="5" t="s">
-        <v>39</v>
-      </c>
     </row>
-    <row r="5" spans="1:16" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>19</v>
       </c>
-      <c r="B5" t="s">
-        <v>30</v>
+      <c r="B5" s="2">
+        <v>46259</v>
       </c>
       <c r="C5" t="s">
         <v>20</v>
@@ -6907,29 +6870,13 @@
         <f t="shared" ca="1" si="1"/>
         <v>Gecikmiş</v>
       </c>
-      <c r="L5" s="6">
-        <f>SUMIFS(G2:G7,I2:I7,"Ödendi")</f>
-        <v>5500</v>
-      </c>
-      <c r="M5" s="7">
-        <f>SUMIFS(G2:G7,I2:I7,"Bekliyor")</f>
-        <v>27000</v>
-      </c>
-      <c r="N5" s="8">
-        <f ca="1">COUNTIFS(H2:H7,"&lt;"&amp;TODAY(),I2:I7,"Bekliyor")</f>
-        <v>3</v>
-      </c>
-      <c r="P5" s="11">
-        <f>SUMIFS(Table1[Toplam_Tutar],Table1[Odeme_Durumu],"Ödendi")/SUM(Table1[Toplam_Tutar])</f>
-        <v>0.16923076923076924</v>
-      </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>22</v>
       </c>
-      <c r="B6" t="s">
-        <v>31</v>
+      <c r="B6" s="2">
+        <v>46261</v>
       </c>
       <c r="C6" t="s">
         <v>9</v>
@@ -6962,12 +6909,12 @@
         <v>Kapandı</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>23</v>
       </c>
-      <c r="B7" t="s">
-        <v>32</v>
+      <c r="B7" s="2">
+        <v>46262</v>
       </c>
       <c r="C7" t="s">
         <v>24</v>

</xml_diff>